<commit_message>
✨ Add HKU karaoke group
</commit_message>
<xml_diff>
--- a/宣群资料/信息.xlsx
+++ b/宣群资料/信息.xlsx
@@ -312,7 +312,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:N16" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:N17" headerRowCount="1">
   <tableColumns count="12">
     <tableColumn id="2" name="Email address"/>
     <tableColumn id="5" name="申请人微信昵称"/>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="18.81640625" customWidth="1" min="3" max="4"/>
@@ -1389,6 +1389,59 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>qr 头图</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>HKU K聚社</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>oliverliu2205@gmail.com</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>星星的猹</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1765386358</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>微信群</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>综合闲聊 / 吹水联络, 唱K，K聚</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>同意入驻，支持 ACA 活动宣传</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>组织jpop、anisongk聚活动，讨论日本流行音乐</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>自我唱功爆上↑↑🎤的同学们注意了⚠️，加入我们hku k聚社摆脱solok无人分担房费的烦恼。我们会不定期举办各种类的jpop、anisong k聚，（如ヨルシカonly、bangdream only等等），也欢迎群友在群里自行组局唱喜欢的歌哦！
+ps:因为k聚绝大多数是日语歌，所以有五十音基础体验会更佳哦</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId1"/>

</xml_diff>